<commit_message>
reran models with data up to 07/2025
</commit_message>
<xml_diff>
--- a/Models/Верблюды/results/Верблюды - Результаты прогнозов Prophet средние.xlsx
+++ b/Models/Верблюды/results/Верблюды - Результаты прогнозов Prophet средние.xlsx
@@ -471,13 +471,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13.02</v>
+        <v>22.66</v>
       </c>
       <c r="C3" t="n">
-        <v>10.63</v>
+        <v>19.19</v>
       </c>
       <c r="D3" t="n">
-        <v>9.01</v>
+        <v>11.96</v>
       </c>
     </row>
     <row r="4">
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54.35</v>
+        <v>50.19</v>
       </c>
       <c r="C4" t="n">
-        <v>40.27</v>
+        <v>36.96</v>
       </c>
       <c r="D4" t="n">
-        <v>328.09</v>
+        <v>326.4</v>
       </c>
     </row>
     <row r="5">
@@ -503,13 +503,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>135.06</v>
+        <v>227.59</v>
       </c>
       <c r="C5" t="n">
-        <v>110.55</v>
+        <v>171.11</v>
       </c>
       <c r="D5" t="n">
-        <v>24.34</v>
+        <v>28.43</v>
       </c>
     </row>
     <row r="6">
@@ -519,10 +519,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.29</v>
+        <v>0.74</v>
       </c>
       <c r="C6" t="n">
-        <v>0.17</v>
+        <v>0.52</v>
       </c>
       <c r="D6" t="inlineStr"/>
     </row>
@@ -575,13 +575,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15.5</v>
+        <v>17.19</v>
       </c>
       <c r="C10" t="n">
-        <v>12.07</v>
+        <v>13.13</v>
       </c>
       <c r="D10" t="n">
-        <v>35.17</v>
+        <v>39.58</v>
       </c>
     </row>
     <row r="11">
@@ -591,13 +591,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5.12</v>
+        <v>4.19</v>
       </c>
       <c r="C11" t="n">
-        <v>4.23</v>
+        <v>3.58</v>
       </c>
       <c r="D11" t="n">
-        <v>50.79</v>
+        <v>47.04</v>
       </c>
     </row>
     <row r="12">
@@ -607,10 +607,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.92</v>
+        <v>4.16</v>
       </c>
       <c r="C12" t="n">
-        <v>3.42</v>
+        <v>3.01</v>
       </c>
       <c r="D12" t="inlineStr"/>
     </row>
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.21</v>
       </c>
       <c r="C13" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="D13" t="inlineStr"/>
     </row>
@@ -635,13 +635,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>766.01</v>
+        <v>1122.56</v>
       </c>
       <c r="C14" t="n">
-        <v>616.12</v>
+        <v>986.02</v>
       </c>
       <c r="D14" t="n">
-        <v>1073.73</v>
+        <v>306.88</v>
       </c>
     </row>
     <row r="15">
@@ -651,13 +651,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>130.37</v>
+        <v>146.75</v>
       </c>
       <c r="C15" t="n">
-        <v>102.98</v>
+        <v>116.67</v>
       </c>
       <c r="D15" t="n">
-        <v>29.31</v>
+        <v>33.17</v>
       </c>
     </row>
     <row r="16">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8803189.17</v>
+        <v>8803222.949999999</v>
       </c>
       <c r="C16" t="n">
-        <v>5082524.25</v>
+        <v>5082544.6</v>
       </c>
       <c r="D16" t="inlineStr"/>
     </row>
@@ -681,10 +681,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>82495870.93000001</v>
+        <v>74061576.87</v>
       </c>
       <c r="C17" t="n">
-        <v>47629157.88</v>
+        <v>42759488.72</v>
       </c>
       <c r="D17" t="inlineStr"/>
     </row>
@@ -695,10 +695,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>213614.59</v>
+        <v>244699.29</v>
       </c>
       <c r="C18" t="n">
-        <v>123330.44</v>
+        <v>141277.2</v>
       </c>
       <c r="D18" t="inlineStr"/>
     </row>
@@ -709,10 +709,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
       <c r="C19" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="D19" t="inlineStr"/>
     </row>
@@ -737,13 +737,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>52.48</v>
+        <v>93.73</v>
       </c>
       <c r="C21" t="n">
-        <v>41.22</v>
+        <v>63.03</v>
       </c>
       <c r="D21" t="n">
-        <v>23.38</v>
+        <v>17.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>